<commit_message>
Fix notebook stream output format; refresh query Excel and JSON
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/evaluation/potential_queries_type_1_2_5_6.xlsx
+++ b/data/evaluation/potential_queries_type_1_2_5_6.xlsx
@@ -4371,12 +4371,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>["EU MARE vessel Russia", "EU MARE ship Russia", "EU MARE vessel RU"]</t>
+          <t>["SECO UKRAINE vessel Russia", "SECO UKRAINE ship Russia", "SECO UKRAINE vessel RU"]</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>programId=EU-MARE | schema=Vessel | country=ru</t>
+          <t>programId=SECO-UKRAINE | schema=Vessel | country=ru</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -4396,12 +4396,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>["SECO UKRAINE vessel Russia", "SECO UKRAINE ship Russia", "SECO UKRAINE vessel RU"]</t>
+          <t>["EU MARE vessel Russia", "EU MARE ship Russia", "EU MARE vessel RU"]</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>programId=SECO-UKRAINE | schema=Vessel | country=ru</t>
+          <t>programId=EU-MARE | schema=Vessel | country=ru</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">

</xml_diff>